<commit_message>
updated splan and cfs #1140
</commit_message>
<xml_diff>
--- a/assets/misc/2026/2026_Attendance2.xlsx
+++ b/assets/misc/2026/2026_Attendance2.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30026"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Documents\git\sqlsatwebsite\assets\misc\2026\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B8CA8CA2-5CF4-4358-A935-06F1822B485F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{294265CB-A082-4DB0-B601-D896D0C8A475}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-23010" yWindow="2475" windowWidth="21330" windowHeight="11280" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="990" yWindow="435" windowWidth="27090" windowHeight="15315" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Attendance" sheetId="1" r:id="rId1"/>
@@ -233,7 +233,7 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="43" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -279,7 +279,6 @@
     <xf numFmtId="3" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="3">
@@ -852,14 +851,14 @@
         <v>28</v>
       </c>
       <c r="C14" s="6">
-        <v>0</v>
+        <v>36</v>
       </c>
       <c r="D14" s="6">
-        <v>0</v>
+        <v>25</v>
       </c>
       <c r="E14" s="7">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>0.30555555555555558</v>
       </c>
     </row>
     <row r="15" spans="1:9" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -1152,28 +1151,28 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A1" s="19" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="19" t="s">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="19" t="s">
+      <c r="C1" t="s">
         <v>22</v>
       </c>
-      <c r="D1" s="19" t="s">
+      <c r="D1" t="s">
         <v>21</v>
       </c>
-      <c r="E1" s="19" t="s">
+      <c r="E1" t="s">
         <v>23</v>
       </c>
-      <c r="F1" s="19" t="s">
+      <c r="F1" t="s">
         <v>24</v>
       </c>
-      <c r="G1" s="19" t="s">
+      <c r="G1" t="s">
         <v>25</v>
       </c>
-      <c r="H1" s="19" t="s">
+      <c r="H1" t="s">
         <v>26</v>
       </c>
     </row>
@@ -1186,16 +1185,16 @@
         <f>+Attendance!B2</f>
         <v>SQL Saturday Lima 2026 (#1138)</v>
       </c>
-      <c r="C2" s="20">
+      <c r="C2" s="19">
         <v>42</v>
       </c>
-      <c r="D2" s="20">
-        <v>0</v>
-      </c>
-      <c r="E2" s="20">
+      <c r="D2" s="19">
+        <v>0</v>
+      </c>
+      <c r="E2" s="19">
         <v>68</v>
       </c>
-      <c r="F2" s="20">
+      <c r="F2" s="19">
         <v>0</v>
       </c>
       <c r="G2" s="8">
@@ -1216,16 +1215,16 @@
         <f>+Attendance!B3</f>
         <v>SQL Saturday Atlanta 2026 - AI &amp; BI (#1127)</v>
       </c>
-      <c r="C3" s="20">
-        <v>0</v>
-      </c>
-      <c r="D3" s="20">
-        <v>0</v>
-      </c>
-      <c r="E3" s="20">
-        <v>0</v>
-      </c>
-      <c r="F3" s="20">
+      <c r="C3" s="19">
+        <v>0</v>
+      </c>
+      <c r="D3" s="19">
+        <v>0</v>
+      </c>
+      <c r="E3" s="19">
+        <v>0</v>
+      </c>
+      <c r="F3" s="19">
         <v>0</v>
       </c>
       <c r="G3" s="8">
@@ -1246,16 +1245,16 @@
         <f>+Attendance!B4</f>
         <v>SQL Saturday Sao Paulo 2026 (#1142)</v>
       </c>
-      <c r="C4" s="20">
+      <c r="C4" s="19">
         <v>28</v>
       </c>
-      <c r="D4" s="20">
+      <c r="D4" s="19">
         <v>5</v>
       </c>
-      <c r="E4" s="20">
+      <c r="E4" s="19">
         <v>46</v>
       </c>
-      <c r="F4" s="20">
+      <c r="F4" s="19">
         <v>8</v>
       </c>
       <c r="G4" s="8">
@@ -1276,16 +1275,16 @@
         <f>+Attendance!B5</f>
         <v>SQL Saturday Joinville 2026 (#1139)</v>
       </c>
-      <c r="C5" s="20">
+      <c r="C5" s="19">
         <v>29</v>
       </c>
-      <c r="D5" s="20">
-        <v>0</v>
-      </c>
-      <c r="E5" s="20">
+      <c r="D5" s="19">
+        <v>0</v>
+      </c>
+      <c r="E5" s="19">
         <v>16</v>
       </c>
-      <c r="F5" s="20">
+      <c r="F5" s="19">
         <v>19</v>
       </c>
       <c r="G5" s="8">
@@ -1548,24 +1547,23 @@
         <v>Day of Data Wellington 2026 (#1146)</v>
       </c>
       <c r="C14">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="D14">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="E14">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="F14">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="G14" s="8">
-        <f t="shared" si="3"/>
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="H14" s="8">
         <f>+Attendance!C14</f>
-        <v>0</v>
+        <v>36</v>
       </c>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
updated splan and cfs #1140 (#1380)
* updated splan and cfs #1140

* update second splan link

---------

Co-authored-by: way0utwest <admin@sqlsaturday.com>
</commit_message>
<xml_diff>
--- a/assets/misc/2026/2026_Attendance2.xlsx
+++ b/assets/misc/2026/2026_Attendance2.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30026"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Documents\git\sqlsatwebsite\assets\misc\2026\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B8CA8CA2-5CF4-4358-A935-06F1822B485F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{294265CB-A082-4DB0-B601-D896D0C8A475}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-23010" yWindow="2475" windowWidth="21330" windowHeight="11280" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="990" yWindow="435" windowWidth="27090" windowHeight="15315" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Attendance" sheetId="1" r:id="rId1"/>
@@ -233,7 +233,7 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="43" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -279,7 +279,6 @@
     <xf numFmtId="3" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="3">
@@ -852,14 +851,14 @@
         <v>28</v>
       </c>
       <c r="C14" s="6">
-        <v>0</v>
+        <v>36</v>
       </c>
       <c r="D14" s="6">
-        <v>0</v>
+        <v>25</v>
       </c>
       <c r="E14" s="7">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>0.30555555555555558</v>
       </c>
     </row>
     <row r="15" spans="1:9" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -1152,28 +1151,28 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A1" s="19" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="19" t="s">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="19" t="s">
+      <c r="C1" t="s">
         <v>22</v>
       </c>
-      <c r="D1" s="19" t="s">
+      <c r="D1" t="s">
         <v>21</v>
       </c>
-      <c r="E1" s="19" t="s">
+      <c r="E1" t="s">
         <v>23</v>
       </c>
-      <c r="F1" s="19" t="s">
+      <c r="F1" t="s">
         <v>24</v>
       </c>
-      <c r="G1" s="19" t="s">
+      <c r="G1" t="s">
         <v>25</v>
       </c>
-      <c r="H1" s="19" t="s">
+      <c r="H1" t="s">
         <v>26</v>
       </c>
     </row>
@@ -1186,16 +1185,16 @@
         <f>+Attendance!B2</f>
         <v>SQL Saturday Lima 2026 (#1138)</v>
       </c>
-      <c r="C2" s="20">
+      <c r="C2" s="19">
         <v>42</v>
       </c>
-      <c r="D2" s="20">
-        <v>0</v>
-      </c>
-      <c r="E2" s="20">
+      <c r="D2" s="19">
+        <v>0</v>
+      </c>
+      <c r="E2" s="19">
         <v>68</v>
       </c>
-      <c r="F2" s="20">
+      <c r="F2" s="19">
         <v>0</v>
       </c>
       <c r="G2" s="8">
@@ -1216,16 +1215,16 @@
         <f>+Attendance!B3</f>
         <v>SQL Saturday Atlanta 2026 - AI &amp; BI (#1127)</v>
       </c>
-      <c r="C3" s="20">
-        <v>0</v>
-      </c>
-      <c r="D3" s="20">
-        <v>0</v>
-      </c>
-      <c r="E3" s="20">
-        <v>0</v>
-      </c>
-      <c r="F3" s="20">
+      <c r="C3" s="19">
+        <v>0</v>
+      </c>
+      <c r="D3" s="19">
+        <v>0</v>
+      </c>
+      <c r="E3" s="19">
+        <v>0</v>
+      </c>
+      <c r="F3" s="19">
         <v>0</v>
       </c>
       <c r="G3" s="8">
@@ -1246,16 +1245,16 @@
         <f>+Attendance!B4</f>
         <v>SQL Saturday Sao Paulo 2026 (#1142)</v>
       </c>
-      <c r="C4" s="20">
+      <c r="C4" s="19">
         <v>28</v>
       </c>
-      <c r="D4" s="20">
+      <c r="D4" s="19">
         <v>5</v>
       </c>
-      <c r="E4" s="20">
+      <c r="E4" s="19">
         <v>46</v>
       </c>
-      <c r="F4" s="20">
+      <c r="F4" s="19">
         <v>8</v>
       </c>
       <c r="G4" s="8">
@@ -1276,16 +1275,16 @@
         <f>+Attendance!B5</f>
         <v>SQL Saturday Joinville 2026 (#1139)</v>
       </c>
-      <c r="C5" s="20">
+      <c r="C5" s="19">
         <v>29</v>
       </c>
-      <c r="D5" s="20">
-        <v>0</v>
-      </c>
-      <c r="E5" s="20">
+      <c r="D5" s="19">
+        <v>0</v>
+      </c>
+      <c r="E5" s="19">
         <v>16</v>
       </c>
-      <c r="F5" s="20">
+      <c r="F5" s="19">
         <v>19</v>
       </c>
       <c r="G5" s="8">
@@ -1548,24 +1547,23 @@
         <v>Day of Data Wellington 2026 (#1146)</v>
       </c>
       <c r="C14">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="D14">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="E14">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="F14">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="G14" s="8">
-        <f t="shared" si="3"/>
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="H14" s="8">
         <f>+Attendance!C14</f>
-        <v>0</v>
+        <v>36</v>
       </c>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.25">

</xml_diff>